<commit_message>
change matrix to custom
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\blob_mechanical\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\VirtualPets\VirtualBlob\Mechanical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8B39E0-C1E1-4E24-8A48-3055D0039C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70105CD-20D8-49F9-A1DF-F5FC1EA1529E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>Name</t>
   </si>
@@ -52,6 +52,12 @@
   </si>
   <si>
     <t>matrix_size</t>
+  </si>
+  <si>
+    <t>shell_width</t>
+  </si>
+  <si>
+    <t>mounting_ratio</t>
   </si>
 </sst>
 </file>
@@ -369,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" customWidth="1"/>
@@ -406,7 +412,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
@@ -432,6 +438,28 @@
       </c>
       <c r="C5" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>0.2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>